<commit_message>
test for submit product review done
</commit_message>
<xml_diff>
--- a/test_scenarios.xlsx
+++ b/test_scenarios.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Login" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="TEST_CASES" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="47">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -151,11 +151,46 @@
     <t xml:space="preserve">1. click on Products
 2. type product name 
 3. click on search button
-4. check searched properly  
-5. check product name present</t>
+4. check searched properly  based on assert</t>
   </si>
   <si>
     <t xml:space="preserve">P2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">search product then view product</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. click on Products
+2. type product name 
+3. click on search button
+4. check searched properly  based on assert
+5. click on specific product’s view product
+6. validate if landed to product details page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">submit review of product</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.open application URL(https://automationexercise.com/)
+2. land to specific product details page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.TC_5 test case should be completed
+2. so once landed to product details page, fill details
+3. submit
+4. validate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P3</t>
   </si>
 </sst>
 </file>
@@ -165,7 +200,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -204,6 +239,12 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -269,7 +310,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -311,6 +352,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -497,12 +542,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="23.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="40.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="51.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="29.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="21.43"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="11.53"/>
@@ -685,7 +731,7 @@
     </row>
     <row r="9" s="8" customFormat="true" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="9" t="s">
         <v>33</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -713,13 +759,67 @@
         <v>16</v>
       </c>
     </row>
+    <row r="11" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="4:4"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="7:7"/>
     <mergeCell ref="9:9"/>
+    <mergeCell ref="12:12"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="1. open application URL(https://automationexercise.com/)&#10;2. should have existing account credentials"/>
@@ -730,6 +830,7 @@
     <hyperlink ref="D6" r:id="rId6" display="1.open application URL(https://automationexercise.com/)"/>
     <hyperlink ref="D8" r:id="rId7" display="1.open application URL(https://automationexercise.com/)"/>
     <hyperlink ref="D10" r:id="rId8" display="1.open application URL(https://automationexercise.com/)"/>
+    <hyperlink ref="D13" r:id="rId9" display="https://automationexercise.com/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>